<commit_message>
chore: update glossary exports
</commit_message>
<xml_diff>
--- a/exports/xlsx/terms_definition_3.xlsx
+++ b/exports/xlsx/terms_definition_3.xlsx
@@ -456,10 +456,98 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ancillary Data</t>
+          <t>Verification</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Evaluation of data reliability in the absence of a reference dataset, confirming consistency and internal coherence.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>- KCEO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Assurance that a product, service, or system meets customer and stakeholder needs through acceptance and suitability evaluation.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>- In this part of ISO 19159, the term validation is used in a limited sense and only relates to the validation of calibration data in order to control their change over time.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>- EU-US Land Imaging EO Collaboration</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Uncertainty</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Measure of the spread of the distribution of possible values.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>- [FIDUCEO Glossary](https://research.reading.ac.uk/fiduceo/glossary/), VIM?, modified</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Auxiliary Data</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>- core
 - to be approved
@@ -468,19 +556,76 @@
 - WGCV</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Data required for instrument processing that does not originate in the instrument itself or from the satellite. Some Auxiliary Data will be generated in the ground segment, whilst other Data will be provided from external sources.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>- CEOS-ARD PFS template 20220302</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>- base
+- to be approved
+- calval ingest
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Property of a phenomenon, body, or substance with a magnitude expressible as a number and a reference.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>- CEOS CalVal Portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ancillary Data</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Data not from the sensor, provided in science telemetry, used to process instrument data and including spacecraft engineering, housekeeping, or subsystem parameters.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>OASIS equivalent definition is ancillary data can be considered as a Digital Data Object (object composed of a set of bit sequences) part of a Content Information, related to other digital objects (i.e. Primary Data) through Context Information (the information that documents the relationships of the Content Information to its environment; this includes why the Content Information was created and how it relates to other Content Information objects) or as a compound digital object which contains a mixture of Provenance, Context and Representation Information related to a Primary Digital Data Object</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
         <is>
           <t>- [CEOS/WGISS/DSIG/GLOS](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)
 - [CEOS-WGISS Document: Auxiliary Data in the CEOS Community: Reference Guidelines Document Part 1: Current Usage (1996) accessible at wgiss.ceos.org/archive/archive.doc/ads200part1.doc](https://calvalportal.ceos.org/web/guest/t-d_wiki?p_p_id=com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn&amp;p_p_lifecycle=0&amp;p_p_state=normal&amp;p_p_mode=view&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_mvcRenderCommandName=%2Fwiki%2Fedit_page&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_redirect=https%3A%2F%2Fcalvalportal.ceos.org%2Fweb%2Fguest%2Ft-d_wiki%3Fp_p_id%3Dcom_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn%26p_p_lifecycle%3D0%26p_p_state%3Dnormal%26p_p_mode%3Dview%26_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_mvcRenderCommandName%3D%252Fwiki%252Fview_page%26_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_nodeName%3DCEOS_Terms_and_Definitions%26_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_title%3DAncillary%2BData&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_nodeId=668236&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_title=CEOS-WGISS+Document%3A+Auxiliary+Data+in+the+CEOS+Community%3A+Reference+Guidelines+Document+Part+1%3A+Current+Usage+%281996%29+accessible+at+wgiss.ceos.org%2Farchive%2Farchive.doc%2Fads200part1.doc)
@@ -489,13 +634,13 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Verification</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Instrument Data</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>- core
 - to be approved
@@ -504,170 +649,21 @@
 - WGISS</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Evaluation of data reliability in the absence of a reference dataset, confirming consistency and internal coherence.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>- KCEO</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Validation</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>- core
-- to be approved
-- calval ingest
-- WGCV
-- WGClimate</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Assurance that a product, service, or system meets customer and stakeholder needs through acceptance and suitability evaluation.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>- In this part of ISO 19159, the term validation is used in a limited sense and only relates to the validation of calibration data in order to control their change over time.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>- EU-US Land Imaging EO Collaboration</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Uncertainty</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>- core
-- to be approved
-- calval ingest
-- WGCV
-- WGISS</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Measure of the spread of the distribution of possible values.</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>- [FIDUCEO Glossary](https://research.reading.ac.uk/fiduceo/glossary/), VIM?, modified</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Instrument Data</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>- core
-- to be approved
-- calval ingest
-- WGCV
-- WGClimate</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Sensor Data, Sensor Data Record</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Data produced and transmitted by the science and engineering sensors of an instrument, and, in the spacecraft environment, any additional data packaged with the instrument's sensor data by virtue of services provided.</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>- [EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Auxiliary Data</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>- core
-- to be approved
-- calval ingest
-- WGCV
-- WGClimate</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Data required for instrument processing that does not originate in the instrument itself or from the satellite. Some Auxiliary Data will be generated in the ground segment, whilst other Data will be provided from external sources.</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>- CEOS-ARD PFS template 20220302</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>- base
-- to be approved
-- calval ingest
-- WGISS
-- WGCV</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Property of a phenomenon, body, or substance with a magnitude expressible as a number and a reference.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>- CEOS CalVal Portal</t>
+          <t>- [EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
         </is>
       </c>
     </row>

</xml_diff>